<commit_message>
feat: updates to preferences
</commit_message>
<xml_diff>
--- a/new_data.xlsx
+++ b/new_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adithya/Documents/neu/Projects/Project_Group_Creator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B851B77-2D67-3B46-B49D-9B9C02E9EF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5636F354-5FC4-694F-8E0B-B29713CA433B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sec 1" sheetId="1" r:id="rId1"/>
@@ -21,24 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="321">
-  <si>
-    <t>Do you already have any specific project ideas? If so, please briefly describe them. (Max 2 ideas)</t>
-  </si>
-  <si>
-    <t>What times during the week can you commit to spending with your group working on the project? 
-(E.g., weekday evenings, weekend mornings, etc)</t>
-  </si>
-  <si>
-    <t>How would you like your group to distribute work over the semester?</t>
-  </si>
-  <si>
-    <t>Are you open to working with, and mentoring students who are new to AI?
-(If you are new to AI, please leave this question blank.)</t>
-  </si>
-  <si>
-    <t>Are there any students in the class you prefer NOT to work with? No reasoning required.†</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="315">
   <si>
     <t>Robotics, Internet of things</t>
   </si>
@@ -1059,9 +1042,6 @@
   </si>
   <si>
     <t>I would like to work with others who are new to AI and are interested in games or finance or robotics</t>
-  </si>
-  <si>
-    <t>Domains of Interest</t>
   </si>
   <si>
     <t>No preference</t>
@@ -2013,27 +1993,27 @@
     <col min="7" max="7" width="255.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>3</v>
+        <v>313</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>4</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -2041,19 +2021,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G2" s="3"/>
     </row>
@@ -2062,16 +2042,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -2081,16 +2061,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -2100,14 +2080,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -2117,14 +2097,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -2134,16 +2114,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -2153,16 +2133,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -2172,16 +2152,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -2191,16 +2171,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -2210,16 +2190,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -2229,14 +2209,14 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -2246,14 +2226,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -2263,16 +2243,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -2282,16 +2262,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -2301,16 +2281,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -2320,14 +2300,14 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
@@ -2337,14 +2317,14 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -2354,17 +2334,17 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G19" s="3"/>
     </row>
@@ -2373,14 +2353,14 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -2390,14 +2370,14 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -2407,16 +2387,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -2426,14 +2406,14 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -2443,14 +2423,14 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -2460,16 +2440,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3">
@@ -2481,16 +2461,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -2500,19 +2480,19 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G27" s="3"/>
     </row>
@@ -2521,16 +2501,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -2540,16 +2520,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -2559,16 +2539,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
@@ -2578,14 +2558,14 @@
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -2595,17 +2575,17 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G32" s="3"/>
     </row>
@@ -2614,17 +2594,17 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G33" s="3"/>
     </row>
@@ -2633,14 +2613,14 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -2650,16 +2630,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -2669,16 +2649,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -2688,16 +2668,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -2707,16 +2687,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -2726,14 +2706,14 @@
         <v>38</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="4" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -2743,20 +2723,20 @@
         <v>39</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2764,14 +2744,14 @@
         <v>40</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -2781,16 +2761,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -2800,16 +2780,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -2819,16 +2799,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -2838,16 +2818,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -2857,20 +2837,20 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -2878,14 +2858,14 @@
         <v>46</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -2895,19 +2875,19 @@
         <v>47</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G48" s="3"/>
     </row>
@@ -2916,17 +2896,17 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G49" s="3"/>
     </row>
@@ -2935,19 +2915,19 @@
         <v>49</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G50" s="3"/>
     </row>
@@ -2956,14 +2936,14 @@
         <v>50</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -2973,16 +2953,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -2992,14 +2972,14 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -3009,16 +2989,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -3028,16 +3008,16 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -3047,16 +3027,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -3066,16 +3046,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -3085,16 +3065,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
@@ -3104,14 +3084,14 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
@@ -3121,16 +3101,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -3155,25 +3135,25 @@
   <sheetData>
     <row r="1" spans="1:7" ht="65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>315</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>318</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -3181,14 +3161,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -3198,14 +3178,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -3215,16 +3195,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -3234,16 +3214,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -3253,14 +3233,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -3270,14 +3250,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -3287,14 +3267,14 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -3304,16 +3284,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -3323,16 +3303,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -3342,16 +3322,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -3361,16 +3341,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -3380,17 +3360,17 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G13" s="3"/>
     </row>
@@ -3399,16 +3379,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -3418,16 +3398,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -3437,16 +3417,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -3456,20 +3436,20 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -3477,16 +3457,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -3496,17 +3476,17 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G19" s="3"/>
     </row>
@@ -3515,16 +3495,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -3534,16 +3514,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -3553,16 +3533,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -3572,16 +3552,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -3591,16 +3571,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -3610,16 +3590,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -3629,19 +3609,19 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G26" s="3"/>
     </row>
@@ -3650,16 +3630,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -3669,16 +3649,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -3688,14 +3668,14 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -3705,20 +3685,20 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="119" x14ac:dyDescent="0.2">
@@ -3726,16 +3706,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -3745,19 +3725,19 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G32" s="3"/>
     </row>
@@ -3766,17 +3746,17 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G33" s="3"/>
     </row>
@@ -3785,17 +3765,17 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G34" s="3"/>
     </row>
@@ -3804,19 +3784,19 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G35" s="3"/>
     </row>
@@ -3825,19 +3805,19 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G36" s="3"/>
     </row>
@@ -3846,16 +3826,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -3865,18 +3845,18 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -3884,19 +3864,19 @@
         <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G39" s="3"/>
     </row>
@@ -3905,16 +3885,16 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -3924,14 +3904,14 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -3941,16 +3921,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -3960,14 +3940,14 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -3977,19 +3957,19 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G44" s="3"/>
     </row>
@@ -3998,16 +3978,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -4017,20 +3997,20 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -4038,14 +4018,14 @@
         <v>46</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -4055,16 +4035,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -4074,16 +4054,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -4093,16 +4073,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -4112,16 +4092,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -4131,19 +4111,19 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G52" s="3"/>
     </row>
@@ -4152,22 +4132,22 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -4175,16 +4155,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -4194,14 +4174,14 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -4211,14 +4191,14 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C56" s="3"/>
       <c r="D56" s="3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -4228,14 +4208,14 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C57" s="3"/>
       <c r="D57" s="3" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -4245,16 +4225,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
@@ -4264,16 +4244,16 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
@@ -4283,16 +4263,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -4302,16 +4282,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -4321,14 +4301,14 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
@@ -4338,19 +4318,19 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G63" s="3"/>
     </row>
@@ -4359,16 +4339,16 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="3"/>
@@ -4378,16 +4358,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
@@ -4397,20 +4377,20 @@
         <v>65</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="3" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
@@ -4418,16 +4398,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -4437,20 +4417,20 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="3" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
@@ -4458,16 +4438,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -4477,16 +4457,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -4496,16 +4476,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -4515,16 +4495,16 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>

</xml_diff>